<commit_message>
Remove feedback entry from defect log
</commit_message>
<xml_diff>
--- a/parcelX/outputs/defectlogs/DefectLogs_Functional_Defects.xlsx
+++ b/parcelX/outputs/defectlogs/DefectLogs_Functional_Defects.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Defects" sheetId="1" r:id="R14f0a369c15c44e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Defects" sheetId="1" r:id="R0e3d36e362194afc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,9 +13,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="@"/>
-  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -47,7 +44,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -66,54 +63,16 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="ECFDF5"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FEF2F2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="92400E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFBEB"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FunctionalDefectLog" displayName="FunctionalDefectLog" ref="A1:P8" headerRowCount="1">
-  <x:autoFilter ref="A1:P8"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FunctionalDefectLog" displayName="FunctionalDefectLog" ref="A1:P7" headerRowCount="1">
+  <x:autoFilter ref="A1:P7"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Module / Feature"/>
     <x:tableColumn id="2" name="Defect ID"/>
@@ -396,10 +355,10 @@
       <x:c r="M2" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N2" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O2" s="8" t="str">
+      <x:c r="N2" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O2" s="7" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P2" s="7" t="str">
@@ -448,10 +407,10 @@
       <x:c r="M3" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N3" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O3" s="8" t="str">
+      <x:c r="N3" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O3" s="7" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P3" s="7" t="str">
@@ -500,10 +459,10 @@
       <x:c r="M4" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N4" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O4" s="8" t="str">
+      <x:c r="N4" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O4" s="7" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P4" s="7" t="str">
@@ -552,10 +511,10 @@
       <x:c r="M5" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N5" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O5" s="8" t="str">
+      <x:c r="N5" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O5" s="7" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P5" s="7" t="str">
@@ -605,10 +564,10 @@
       <x:c r="M6" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N6" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O6" s="8" t="str">
+      <x:c r="N6" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O6" s="7" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P6" s="7" t="str">
@@ -617,129 +576,71 @@
     </x:row>
     <x:row r="7" ht="66" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Feedback</x:v>
+        <x:v>Payment</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
         <x:v>FD-006</x:v>
       </x:c>
       <x:c r="C7" s="7" t="str">
-        <x:v>Refresh button visible in feedback</x:v>
+        <x:v>CVV toggle uses text instead of eye icon</x:v>
       </x:c>
       <x:c r="D7" s="7" t="str">
-        <x:v>Admin feedback</x:v>
+        <x:v>Payment card form</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
-        <x:v>Admin feedback section displayed a refresh button that was not required.</x:v>
+        <x:v>CVV visibility toggle displayed Show and Hide text instead of an eye icon.</x:v>
       </x:c>
       <x:c r="F7" s="7" t="str">
-        <x:v>1. Login as admin.
-2. Open Feedback tab.</x:v>
-      </x:c>
-      <x:c r="G7" s="7" t="str">
-        <x:v>Feedback should show without a refresh button.</x:v>
-      </x:c>
-      <x:c r="H7" s="7" t="str">
-        <x:v>Refresh button was visible in the feedback section.</x:v>
-      </x:c>
-      <x:c r="I7" s="7" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="J7" s="7" t="str">
-        <x:v>P3</x:v>
-      </x:c>
-      <x:c r="K7" s="7" t="str">
-        <x:v>Closed</x:v>
-      </x:c>
-      <x:c r="L7" s="7" t="str">
-        <x:v>Shriharsha K M</x:v>
-      </x:c>
-      <x:c r="M7" s="7" t="str">
-        <x:v>Shriharsha K M</x:v>
-      </x:c>
-      <x:c r="N7" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O7" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="P7" s="7" t="str">
-        <x:v>Visible refresh controls removed from frontend screens.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="66" customHeight="1">
-      <x:c r="A8" s="7" t="str">
-        <x:v>Payment</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="str">
-        <x:v>FD-007</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="str">
-        <x:v>CVV toggle uses text instead of eye icon</x:v>
-      </x:c>
-      <x:c r="D8" s="7" t="str">
-        <x:v>Payment card form</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="str">
-        <x:v>CVV visibility toggle displayed Show and Hide text instead of an eye icon.</x:v>
-      </x:c>
-      <x:c r="F8" s="7" t="str">
         <x:v>1. Open payment page.
 2. Select card payment.
 3. Inspect CVV field visibility toggle.</x:v>
       </x:c>
-      <x:c r="G8" s="7" t="str">
+      <x:c r="G7" s="7" t="str">
         <x:v>CVV field should use an icon-only visibility toggle.</x:v>
       </x:c>
-      <x:c r="H8" s="7" t="str">
+      <x:c r="H7" s="7" t="str">
         <x:v>CVV field used Show and Hide text.</x:v>
       </x:c>
-      <x:c r="I8" s="7" t="str">
+      <x:c r="I7" s="7" t="str">
         <x:v>Low</x:v>
       </x:c>
-      <x:c r="J8" s="7" t="str">
+      <x:c r="J7" s="7" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K8" s="7" t="str">
+      <x:c r="K7" s="7" t="str">
         <x:v>Closed</x:v>
       </x:c>
-      <x:c r="L8" s="7" t="str">
-        <x:v>Shriharsha K M</x:v>
-      </x:c>
-      <x:c r="M8" s="7" t="str">
-        <x:v>Shriharsha K M</x:v>
-      </x:c>
-      <x:c r="N8" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O8" s="8" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="P8" s="7" t="str">
+      <x:c r="L7" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="M7" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="N7" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O7" s="7" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="P7" s="7" t="str">
         <x:v>CVV visibility toggle changed to an eye icon button.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="K2:K8">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I2:I8">
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="High"/>
-  </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="I2:I8">
+    <x:dataValidation type="list" sqref="I2:I7">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J2:J8">
+    <x:dataValidation type="list" sqref="J2:J7">
       <x:formula1>"P1,P2,P3"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K8">
+    <x:dataValidation type="list" sqref="K2:K7">
       <x:formula1>"Open,In Progress,Fixed,Closed"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re934d676c8264ee9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18da86cc6b54046"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate functional defect log
</commit_message>
<xml_diff>
--- a/parcelX/outputs/defectlogs/DefectLogs_Functional_Defects.xlsx
+++ b/parcelX/outputs/defectlogs/DefectLogs_Functional_Defects.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Defects" sheetId="1" r:id="R0e3d36e362194afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional Defects" sheetId="1" r:id="R0a22e3f170054478"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,6 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -44,7 +47,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -63,16 +66,54 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="3">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="ECFDF5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FEF2F2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFBEB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FunctionalDefectLog" displayName="FunctionalDefectLog" ref="A1:P7" headerRowCount="1">
-  <x:autoFilter ref="A1:P7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FunctionalDefectLog" displayName="FunctionalDefectLog" ref="A1:P9" headerRowCount="1">
+  <x:autoFilter ref="A1:P9"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Module / Feature"/>
     <x:tableColumn id="2" name="Defect ID"/>
@@ -245,24 +286,24 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="19.520000457763672" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.770000457763672" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28.940000534057617" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20.860000610351562" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="39.70000076293945" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="39.70000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="34.31999969482422" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="34.31999969482422" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30.280000686645508" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21.530000686645508" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="41.04999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="41.04999923706055" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="35.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="35.66999816894531" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="12.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="10.09000015258789" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="14.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="16.81999969482422" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16.81999969482422" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="13.460000038146973" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="13.460000038146973" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="39.70000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="41.04999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="31.5" customHeight="1">
+    <x:row r="1" ht="33" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>Module / Feature</x:v>
       </x:c>
@@ -312,7 +353,7 @@
         <x:v>Comments / Remarks</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="66" customHeight="1">
+    <x:row r="2" ht="69" customHeight="1">
       <x:c r="A2" s="7" t="str">
         <x:v>Admin Parcel Booking</x:v>
       </x:c>
@@ -320,25 +361,25 @@
         <x:v>FD-001</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Admin cannot book parcel</x:v>
+        <x:v>Admin booking shows access denied</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
         <x:v>Admin booking</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Admin user was blocked from creating a parcel because the parcel booking endpoint allowed only customer access.</x:v>
+        <x:v>The admin parcel booking form could not create a parcel because the backend booking endpoint did not allow admin users.</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>1. Login as admin.
+        <x:v>1. Login with admin credentials.
 2. Open Admin Dashboard.
-3. Go to Book Parcel.
+3. Open Book Parcel.
 4. Submit valid parcel details.</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>Admin should be able to book a parcel from the admin dashboard.</x:v>
+        <x:v>Admin should be able to create a parcel from the admin dashboard.</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Application showed access denied while booking parcel as admin.</x:v>
+        <x:v>The request failed with an access denied response.</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
         <x:v>High</x:v>
@@ -355,17 +396,17 @@
       <x:c r="M2" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N2" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O2" s="7" t="str">
+      <x:c r="N2" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O2" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P2" s="7" t="str">
-        <x:v>Backend parcel booking access updated for admin and customer roles.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="66" customHeight="1">
+        <x:v>Parcel booking access was updated for ADMIN and CUSTOMER users.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="69" customHeight="1">
       <x:c r="A3" s="7" t="str">
         <x:v>Registration</x:v>
       </x:c>
@@ -373,24 +414,24 @@
         <x:v>FD-002</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
-        <x:v>No acknowledgement after registration</x:v>
+        <x:v>Registration completes without acknowledgement</x:v>
       </x:c>
       <x:c r="D3" s="7" t="str">
         <x:v>Customer registration</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>Customer registration completed without a clear acknowledgement message in the UI.</x:v>
+        <x:v>After successful customer registration, the UI did not show a clear acknowledgement message to the user.</x:v>
       </x:c>
       <x:c r="F3" s="7" t="str">
-        <x:v>1. Open registration page.
+        <x:v>1. Open Register.
 2. Enter valid customer details.
-3. Submit registration form.</x:v>
+3. Submit the form.</x:v>
       </x:c>
       <x:c r="G3" s="7" t="str">
-        <x:v>Application should show a registration acknowledgement message.</x:v>
+        <x:v>The application should show a success acknowledgement after registration.</x:v>
       </x:c>
       <x:c r="H3" s="7" t="str">
-        <x:v>Registration completed without an acknowledgement message.</x:v>
+        <x:v>The user was not shown a clear registration acknowledgement.</x:v>
       </x:c>
       <x:c r="I3" s="7" t="str">
         <x:v>Medium</x:v>
@@ -407,17 +448,17 @@
       <x:c r="M3" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N3" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O3" s="7" t="str">
+      <x:c r="N3" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O3" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P3" s="7" t="str">
-        <x:v>Frontend registration acknowledgement modal added.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="66" customHeight="1">
+        <x:v>Registration acknowledgement message was added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="69" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>Admin Users</x:v>
       </x:c>
@@ -425,24 +466,24 @@
         <x:v>FD-003</x:v>
       </x:c>
       <x:c r="C4" s="7" t="str">
-        <x:v>Admin users list fails to load</x:v>
+        <x:v>Admin dashboard fails to load users</x:v>
       </x:c>
       <x:c r="D4" s="7" t="str">
-        <x:v>Admin dashboard users</x:v>
+        <x:v>User management</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
-        <x:v>Admin dashboard displayed failed to load users due to role and authorization handling around user data.</x:v>
+        <x:v>The admin dashboard displayed a failure message while loading registered users.</x:v>
       </x:c>
       <x:c r="F4" s="7" t="str">
-        <x:v>1. Login as admin.
+        <x:v>1. Login with admin credentials.
 2. Open Admin Dashboard.
-3. Go to Users tab.</x:v>
+3. Open Users tab.</x:v>
       </x:c>
       <x:c r="G4" s="7" t="str">
-        <x:v>Admin should see the users list.</x:v>
+        <x:v>Admin should be able to view the users list.</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
-        <x:v>Application showed failed to load users.</x:v>
+        <x:v>The UI showed failed to load users.</x:v>
       </x:c>
       <x:c r="I4" s="7" t="str">
         <x:v>High</x:v>
@@ -459,42 +500,42 @@
       <x:c r="M4" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N4" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O4" s="7" t="str">
+      <x:c r="N4" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O4" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P4" s="7" t="str">
-        <x:v>Role handling kept to ADMIN and CUSTOMER and admin user loading fixed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="66" customHeight="1">
+        <x:v>Admin user loading and role handling were corrected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="69" customHeight="1">
       <x:c r="A5" s="7" t="str">
-        <x:v>Admin Orders</x:v>
+        <x:v>Roles</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
         <x:v>FD-004</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>Admin cannot see payment status</x:v>
+        <x:v>Unsupported delivery-agent role remains in project</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
-        <x:v>Admin dashboard orders</x:v>
+        <x:v>Authorization roles</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
-        <x:v>Admin all-orders view did not show payment status for parcels.</x:v>
+        <x:v>The project contained delivery-agent role references even though only admin and customer roles are required.</x:v>
       </x:c>
       <x:c r="F5" s="7" t="str">
-        <x:v>1. Login as admin.
-2. Open Admin Dashboard.
-3. Go to All Orders.</x:v>
+        <x:v>1. Review login/authorization flows.
+2. Review backend role definitions and protected routes.
+3. Compare available roles with project requirements.</x:v>
       </x:c>
       <x:c r="G5" s="7" t="str">
-        <x:v>Admin should see payment status for each parcel.</x:v>
+        <x:v>The application should support only ADMIN and CUSTOMER roles.</x:v>
       </x:c>
       <x:c r="H5" s="7" t="str">
-        <x:v>Payment status was not visible in the admin orders table and details.</x:v>
+        <x:v>DELIVERY_AGENT references existed in role handling.</x:v>
       </x:c>
       <x:c r="I5" s="7" t="str">
         <x:v>Medium</x:v>
@@ -511,49 +552,49 @@
       <x:c r="M5" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N5" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O5" s="7" t="str">
+      <x:c r="N5" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O5" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P5" s="7" t="str">
-        <x:v>Payment status, method, and transaction details added to admin parcel views.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="66" customHeight="1">
+        <x:v>Role handling was limited to ADMIN and CUSTOMER.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="69" customHeight="1">
       <x:c r="A6" s="7" t="str">
-        <x:v>Admin Status Update</x:v>
+        <x:v>Admin Orders</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
         <x:v>FD-005</x:v>
       </x:c>
       <x:c r="C6" s="7" t="str">
-        <x:v>Admin can change status while payment is pending</x:v>
+        <x:v>Payment status not visible to admin</x:v>
       </x:c>
       <x:c r="D6" s="7" t="str">
-        <x:v>Admin dashboard orders</x:v>
+        <x:v>Admin order management</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
-        <x:v>Admin status dropdown allowed status changes before parcel payment was confirmed.</x:v>
+        <x:v>The admin order views did not show parcel payment status, method, or transaction details.</x:v>
       </x:c>
       <x:c r="F6" s="7" t="str">
-        <x:v>1. Login as admin.
-2. Open All Orders.
-3. Find a parcel with pending payment.
-4. Try changing parcel status.</x:v>
+        <x:v>1. Login with admin credentials.
+2. Open Admin Dashboard.
+3. Open All Orders.
+4. View parcel details.</x:v>
       </x:c>
       <x:c r="G6" s="7" t="str">
-        <x:v>Status update should be blocked until payment is confirmed.</x:v>
+        <x:v>Admin should see payment status and available payment details for parcels.</x:v>
       </x:c>
       <x:c r="H6" s="7" t="str">
-        <x:v>Status could be changed while payment was pending.</x:v>
+        <x:v>Payment information was missing from the admin order views.</x:v>
       </x:c>
       <x:c r="I6" s="7" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="K6" s="7" t="str">
         <x:v>Closed</x:v>
@@ -564,48 +605,49 @@
       <x:c r="M6" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N6" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O6" s="7" t="str">
+      <x:c r="N6" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O6" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P6" s="7" t="str">
-        <x:v>Admin status dropdown is disabled for pending payment and update method is guarded.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="66" customHeight="1">
+        <x:v>Payment status, payment method, and transaction ID display were added to admin views.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="69" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>Payment</x:v>
+        <x:v>Admin Status Update</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
         <x:v>FD-006</x:v>
       </x:c>
       <x:c r="C7" s="7" t="str">
-        <x:v>CVV toggle uses text instead of eye icon</x:v>
+        <x:v>Admin can update parcel status before payment confirmation</x:v>
       </x:c>
       <x:c r="D7" s="7" t="str">
-        <x:v>Payment card form</x:v>
+        <x:v>Admin order status</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
-        <x:v>CVV visibility toggle displayed Show and Hide text instead of an eye icon.</x:v>
+        <x:v>The admin status control allowed status changes even when a parcel payment was still pending.</x:v>
       </x:c>
       <x:c r="F7" s="7" t="str">
-        <x:v>1. Open payment page.
-2. Select card payment.
-3. Inspect CVV field visibility toggle.</x:v>
+        <x:v>1. Login with admin credentials.
+2. Open All Orders.
+3. Locate a parcel with pending payment.
+4. Attempt to change parcel status.</x:v>
       </x:c>
       <x:c r="G7" s="7" t="str">
-        <x:v>CVV field should use an icon-only visibility toggle.</x:v>
+        <x:v>Admin should be blocked from changing status until payment is confirmed.</x:v>
       </x:c>
       <x:c r="H7" s="7" t="str">
-        <x:v>CVV field used Show and Hide text.</x:v>
+        <x:v>Status could be changed before payment confirmation.</x:v>
       </x:c>
       <x:c r="I7" s="7" t="str">
-        <x:v>Low</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
-        <x:v>P3</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="K7" s="7" t="str">
         <x:v>Closed</x:v>
@@ -616,31 +658,141 @@
       <x:c r="M7" s="7" t="str">
         <x:v>Shriharsha K M</x:v>
       </x:c>
-      <x:c r="N7" s="7" t="str">
-        <x:v>2026-05-10</x:v>
-      </x:c>
-      <x:c r="O7" s="7" t="str">
+      <x:c r="N7" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O7" s="8" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="P7" s="7" t="str">
-        <x:v>CVV visibility toggle changed to an eye icon button.</x:v>
+        <x:v>Status dropdown was disabled for unpaid parcels and update logic was guarded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="69" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>Payment</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>FD-007</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="str">
+        <x:v>CVV visibility control uses text labels</x:v>
+      </x:c>
+      <x:c r="D8" s="7" t="str">
+        <x:v>Card payment form</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="str">
+        <x:v>The CVV visibility control displayed Show and Hide text instead of an icon-only control.</x:v>
+      </x:c>
+      <x:c r="F8" s="7" t="str">
+        <x:v>1. Open the payment page.
+2. Select card payment.
+3. Check the CVV field visibility control.</x:v>
+      </x:c>
+      <x:c r="G8" s="7" t="str">
+        <x:v>The CVV field should use an eye icon control.</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="str">
+        <x:v>The control displayed Show and Hide text labels.</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="J8" s="7" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="K8" s="7" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L8" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="M8" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="N8" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O8" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="P8" s="7" t="str">
+        <x:v>CVV visibility control was changed to an eye icon.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="69" customHeight="1">
+      <x:c r="A9" s="7" t="str">
+        <x:v>Branding</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="str">
+        <x:v>FD-008</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="str">
+        <x:v>Project name is inconsistent in UI</x:v>
+      </x:c>
+      <x:c r="D9" s="7" t="str">
+        <x:v>Application branding</x:v>
+      </x:c>
+      <x:c r="E9" s="7" t="str">
+        <x:v>The visible project name did not match the requested project name across UI screens.</x:v>
+      </x:c>
+      <x:c r="F9" s="7" t="str">
+        <x:v>1. Open landing, login, registration, user, and admin screens.
+2. Check visible project title text.</x:v>
+      </x:c>
+      <x:c r="G9" s="7" t="str">
+        <x:v>Screens should show the requested project name consistently.</x:v>
+      </x:c>
+      <x:c r="H9" s="7" t="str">
+        <x:v>Screens showed the old project name.</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="J9" s="7" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="K9" s="7" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L9" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="M9" s="7" t="str">
+        <x:v>Shriharsha K M</x:v>
+      </x:c>
+      <x:c r="N9" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O9" s="8" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="P9" s="7" t="str">
+        <x:v>Visible project name was updated across frontend screens and documentation.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="K2:K9">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I2:I9">
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="High"/>
+  </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="I2:I7">
+    <x:dataValidation type="list" sqref="I2:I9">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J2:J7">
+    <x:dataValidation type="list" sqref="J2:J9">
       <x:formula1>"P1,P2,P3"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K7">
+    <x:dataValidation type="list" sqref="K2:K9">
       <x:formula1>"Open,In Progress,Fixed,Closed"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18da86cc6b54046"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28f1b99a7d174a3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>